<commit_message>
Make costs consistently per treatment group member
</commit_message>
<xml_diff>
--- a/data/extraction_full_v18.xlsx
+++ b/data/extraction_full_v18.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\drood\Dropbox\Job training meta-analysis\job-training-meta-analysis\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\drood\Dropbox\Job training meta-analysis\job-training-meta-analysis\job-training-meta-analysis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B47728A5-494A-4033-AFB1-15FCADB2BC44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99436704-4D96-4833-B980-6829CCA6F654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1740" yWindow="1740" windowWidth="17280" windowHeight="10524" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="14592" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Table" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data Table'!$A$1:$CJ$145</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -10333,7 +10346,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:CJ145"/>
   <sheetFormatPr defaultRowHeight="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -11539,7 +11551,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="6" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="2" t="s">
         <v>139</v>
       </c>
@@ -11780,7 +11792,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="7" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="2" t="s">
         <v>139</v>
       </c>
@@ -12016,7 +12028,7 @@
         <v>2.8</v>
       </c>
     </row>
-    <row r="8" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="2" t="s">
         <v>139</v>
       </c>
@@ -12246,7 +12258,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="9" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="2" t="s">
         <v>139</v>
       </c>
@@ -12476,7 +12488,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="10" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="2" t="s">
         <v>174</v>
       </c>
@@ -12676,7 +12688,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="11" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="2" t="s">
         <v>174</v>
       </c>
@@ -12882,7 +12894,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="12" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="2" t="s">
         <v>174</v>
       </c>
@@ -13082,7 +13094,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="13" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="2" t="s">
         <v>174</v>
       </c>
@@ -13282,7 +13294,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="14" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="2" t="s">
         <v>174</v>
       </c>
@@ -13482,7 +13494,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="15" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="2" t="s">
         <v>174</v>
       </c>
@@ -13682,7 +13694,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="16" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="2" t="s">
         <v>174</v>
       </c>
@@ -13882,7 +13894,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="17" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="2" t="s">
         <v>174</v>
       </c>
@@ -14082,7 +14094,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="18" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="2" t="s">
         <v>174</v>
       </c>
@@ -14282,7 +14294,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="19" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="2" t="s">
         <v>174</v>
       </c>
@@ -14482,7 +14494,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="20" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="2" t="s">
         <v>174</v>
       </c>
@@ -14682,7 +14694,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="21" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="2" t="s">
         <v>174</v>
       </c>
@@ -14882,7 +14894,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="22" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="2" t="s">
         <v>174</v>
       </c>
@@ -15082,7 +15094,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="23" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="2" t="s">
         <v>233</v>
       </c>
@@ -15289,7 +15301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="2" t="s">
         <v>233</v>
       </c>
@@ -15494,7 +15506,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="25" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="2" t="s">
         <v>233</v>
       </c>
@@ -15697,7 +15709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="2" t="s">
         <v>233</v>
       </c>
@@ -15918,7 +15930,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="27" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="2" t="s">
         <v>233</v>
       </c>
@@ -16139,7 +16151,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="28" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="2" t="s">
         <v>233</v>
       </c>
@@ -16344,7 +16356,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="29" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="2" t="s">
         <v>284</v>
       </c>
@@ -16532,7 +16544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="2" t="s">
         <v>296</v>
       </c>
@@ -16764,7 +16776,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="2" t="s">
         <v>311</v>
       </c>
@@ -16982,7 +16994,7 @@
         <v>35.299999999999997</v>
       </c>
     </row>
-    <row r="32" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="2" t="s">
         <v>311</v>
       </c>
@@ -17200,7 +17212,7 @@
         <v>55.2</v>
       </c>
     </row>
-    <row r="33" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="2" t="s">
         <v>311</v>
       </c>
@@ -17418,7 +17430,7 @@
         <v>47.1</v>
       </c>
     </row>
-    <row r="34" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="2" t="s">
         <v>311</v>
       </c>
@@ -17625,7 +17637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="2" t="s">
         <v>311</v>
       </c>
@@ -17827,7 +17839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="2" t="s">
         <v>311</v>
       </c>
@@ -18031,7 +18043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="2" t="s">
         <v>311</v>
       </c>
@@ -18228,7 +18240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="2" t="s">
         <v>311</v>
       </c>
@@ -18451,7 +18463,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="39" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="2" t="s">
         <v>369</v>
       </c>
@@ -18665,7 +18677,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="40" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="2" t="s">
         <v>369</v>
       </c>
@@ -18870,7 +18882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" s="2" t="s">
         <v>369</v>
       </c>
@@ -19076,7 +19088,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="42" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="2" t="s">
         <v>369</v>
       </c>
@@ -19279,7 +19291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="2" t="s">
         <v>369</v>
       </c>
@@ -19484,7 +19496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="2" t="s">
         <v>369</v>
       </c>
@@ -19684,7 +19696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="2" t="s">
         <v>369</v>
       </c>
@@ -19891,7 +19903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="2" t="s">
         <v>369</v>
       </c>
@@ -20100,7 +20112,7 @@
         <v>2.7</v>
       </c>
     </row>
-    <row r="47" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="2" t="s">
         <v>430</v>
       </c>
@@ -20335,7 +20347,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="2" t="s">
         <v>446</v>
       </c>
@@ -20517,7 +20529,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="2" t="s">
         <v>446</v>
       </c>
@@ -20697,7 +20709,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="50" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="2" t="s">
         <v>446</v>
       </c>
@@ -20878,7 +20890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="2" t="s">
         <v>446</v>
       </c>
@@ -21057,7 +21069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="2" t="s">
         <v>446</v>
       </c>
@@ -21237,7 +21249,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="53" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="2" t="s">
         <v>446</v>
       </c>
@@ -21418,7 +21430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="2" t="s">
         <v>446</v>
       </c>
@@ -21598,7 +21610,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="2" t="s">
         <v>493</v>
       </c>
@@ -21798,7 +21810,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="56" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="2" t="s">
         <v>493</v>
       </c>
@@ -21980,7 +21992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="2" t="s">
         <v>493</v>
       </c>
@@ -22166,7 +22178,7 @@
         <v>33.799999999999997</v>
       </c>
     </row>
-    <row r="58" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="2" t="s">
         <v>493</v>
       </c>
@@ -22368,7 +22380,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="2" t="s">
         <v>493</v>
       </c>
@@ -22568,7 +22580,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="2" t="s">
         <v>493</v>
       </c>
@@ -22753,7 +22765,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="2" t="s">
         <v>552</v>
       </c>
@@ -22989,7 +23001,7 @@
         <v>3.75</v>
       </c>
     </row>
-    <row r="62" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="2" t="s">
         <v>552</v>
       </c>
@@ -23214,7 +23226,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="63" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="2" t="s">
         <v>552</v>
       </c>
@@ -23439,7 +23451,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="64" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="2" t="s">
         <v>552</v>
       </c>
@@ -23672,7 +23684,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="65" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="2" t="s">
         <v>591</v>
       </c>
@@ -23867,7 +23879,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="66" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="2" t="s">
         <v>591</v>
       </c>
@@ -24064,7 +24076,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="67" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="2" t="s">
         <v>591</v>
       </c>
@@ -24261,7 +24273,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="68" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="2" t="s">
         <v>619</v>
       </c>
@@ -24454,7 +24466,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="69" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="2" t="s">
         <v>619</v>
       </c>
@@ -24647,7 +24659,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="70" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="2" t="s">
         <v>619</v>
       </c>
@@ -24842,7 +24854,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="71" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="2" t="s">
         <v>619</v>
       </c>
@@ -25035,7 +25047,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="72" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="72" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" t="s">
         <v>654</v>
       </c>
@@ -25205,7 +25217,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="73" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" t="s">
         <v>654</v>
       </c>
@@ -25378,7 +25390,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="74" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" t="s">
         <v>654</v>
       </c>
@@ -25551,7 +25563,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="75" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" t="s">
         <v>654</v>
       </c>
@@ -25718,7 +25730,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="76" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A76" t="s">
         <v>654</v>
       </c>
@@ -25891,7 +25903,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="77" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A77" t="s">
         <v>654</v>
       </c>
@@ -26061,7 +26073,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="78" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="78" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A78" t="s">
         <v>654</v>
       </c>
@@ -26231,7 +26243,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="79" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="79" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A79" t="s">
         <v>699</v>
       </c>
@@ -26398,7 +26410,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="80" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A80" t="s">
         <v>699</v>
       </c>
@@ -26565,7 +26577,7 @@
         <v>55.7</v>
       </c>
     </row>
-    <row r="81" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="81" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A81" t="s">
         <v>699</v>
       </c>
@@ -26732,7 +26744,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="82" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A82" t="s">
         <v>699</v>
       </c>
@@ -26899,7 +26911,7 @@
         <v>48.6</v>
       </c>
     </row>
-    <row r="83" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="83" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A83" t="s">
         <v>721</v>
       </c>
@@ -27051,7 +27063,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="84" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="84" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A84" t="s">
         <v>721</v>
       </c>
@@ -27203,7 +27215,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="85" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="85" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A85" t="s">
         <v>735</v>
       </c>
@@ -27385,7 +27397,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="86" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="86" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A86" t="s">
         <v>749</v>
       </c>
@@ -27552,7 +27564,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="87" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="87" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A87" t="s">
         <v>763</v>
       </c>
@@ -27731,7 +27743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="88" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="88" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A88" t="s">
         <v>775</v>
       </c>
@@ -27877,7 +27889,7 @@
         <v>12.7</v>
       </c>
     </row>
-    <row r="89" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="89" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A89" t="s">
         <v>787</v>
       </c>
@@ -28086,7 +28098,7 @@
         <v>12.4</v>
       </c>
     </row>
-    <row r="90" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="90" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A90" t="s">
         <v>802</v>
       </c>
@@ -28286,7 +28298,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="91" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="91" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A91" t="s">
         <v>802</v>
       </c>
@@ -28483,7 +28495,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="92" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="92" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A92" t="s">
         <v>825</v>
       </c>
@@ -28698,7 +28710,7 @@
         <v>24.9</v>
       </c>
     </row>
-    <row r="93" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="93" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A93" t="s">
         <v>825</v>
       </c>
@@ -28901,7 +28913,7 @@
         <v>34.200000000000003</v>
       </c>
     </row>
-    <row r="94" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="94" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A94" t="s">
         <v>825</v>
       </c>
@@ -29107,7 +29119,7 @@
         <v>31.9</v>
       </c>
     </row>
-    <row r="95" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="95" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A95" t="s">
         <v>825</v>
       </c>
@@ -29310,7 +29322,7 @@
         <v>31.9</v>
       </c>
     </row>
-    <row r="96" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="96" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A96" t="s">
         <v>825</v>
       </c>
@@ -29513,7 +29525,7 @@
         <v>37.299999999999997</v>
       </c>
     </row>
-    <row r="97" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="97" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A97" t="s">
         <v>825</v>
       </c>
@@ -29716,7 +29728,7 @@
         <v>25.1</v>
       </c>
     </row>
-    <row r="98" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="98" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A98" t="s">
         <v>825</v>
       </c>
@@ -29919,7 +29931,7 @@
         <v>21.6</v>
       </c>
     </row>
-    <row r="99" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="99" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A99" t="s">
         <v>825</v>
       </c>
@@ -30143,7 +30155,7 @@
         <v>39.9</v>
       </c>
     </row>
-    <row r="100" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="100" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A100" t="s">
         <v>901</v>
       </c>
@@ -30301,7 +30313,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="101" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="101" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A101" t="s">
         <v>901</v>
       </c>
@@ -30456,7 +30468,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="102" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="102" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A102" t="s">
         <v>901</v>
       </c>
@@ -30614,7 +30626,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="103" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="103" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A103" t="s">
         <v>901</v>
       </c>
@@ -30775,7 +30787,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="104" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="104" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A104" t="s">
         <v>922</v>
       </c>
@@ -30936,7 +30948,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="105" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="105" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A105" t="s">
         <v>934</v>
       </c>
@@ -31145,7 +31157,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="106" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A106" t="s">
         <v>934</v>
       </c>
@@ -31345,7 +31357,7 @@
         <v>38.1</v>
       </c>
     </row>
-    <row r="107" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="107" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A107" t="s">
         <v>953</v>
       </c>
@@ -31560,7 +31572,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="108" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="108" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A108" t="s">
         <v>967</v>
       </c>
@@ -31727,7 +31739,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="109" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="109" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A109" t="s">
         <v>825</v>
       </c>
@@ -31906,7 +31918,7 @@
         <v>26.3</v>
       </c>
     </row>
-    <row r="110" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="110" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A110" t="s">
         <v>988</v>
       </c>
@@ -32109,7 +32121,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="111" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="111" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A111" t="s">
         <v>1001</v>
       </c>
@@ -32240,7 +32252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="112" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A112" t="s">
         <v>1001</v>
       </c>
@@ -32371,7 +32383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="113" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A113" t="s">
         <v>1001</v>
       </c>
@@ -32511,7 +32523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="114" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A114" t="s">
         <v>1022</v>
       </c>
@@ -32717,7 +32729,7 @@
         <v>26.2</v>
       </c>
     </row>
-    <row r="115" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="115" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A115" t="s">
         <v>1036</v>
       </c>
@@ -32932,7 +32944,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="116" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="116" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A116" t="s">
         <v>1047</v>
       </c>
@@ -33117,7 +33129,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="117" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="117" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A117" t="s">
         <v>1057</v>
       </c>
@@ -33314,7 +33326,7 @@
         <v>53.7</v>
       </c>
     </row>
-    <row r="118" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="118" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A118" t="s">
         <v>1057</v>
       </c>
@@ -33508,7 +33520,7 @@
         <v>44.3</v>
       </c>
     </row>
-    <row r="119" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="119" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A119" t="s">
         <v>1057</v>
       </c>
@@ -33651,7 +33663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="120" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A120" t="s">
         <v>1077</v>
       </c>
@@ -33863,7 +33875,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="121" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="121" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A121" t="s">
         <v>1087</v>
       </c>
@@ -34045,7 +34057,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="122" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="122" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A122" t="s">
         <v>1100</v>
       </c>
@@ -34197,7 +34209,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="123" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="123" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A123" t="s">
         <v>1111</v>
       </c>
@@ -34361,7 +34373,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="124" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="124" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A124" t="s">
         <v>1122</v>
       </c>
@@ -34579,7 +34591,7 @@
         <v>49.6</v>
       </c>
     </row>
-    <row r="125" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="125" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A125" t="s">
         <v>1134</v>
       </c>
@@ -34722,7 +34734,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="126" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="126" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A126" t="s">
         <v>1146</v>
       </c>
@@ -34895,7 +34907,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="127" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="127" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A127" t="s">
         <v>1157</v>
       </c>
@@ -35104,7 +35116,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="128" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="128" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A128" t="s">
         <v>1157</v>
       </c>
@@ -35307,7 +35319,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="129" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="129" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A129" t="s">
         <v>1174</v>
       </c>
@@ -35474,7 +35486,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="130" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="130" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A130" t="s">
         <v>1186</v>
       </c>
@@ -35665,7 +35677,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="131" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="131" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A131" t="s">
         <v>1198</v>
       </c>
@@ -35787,7 +35799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="132" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A132" t="s">
         <v>1209</v>
       </c>
@@ -35954,7 +35966,7 @@
         <v>66.900000000000006</v>
       </c>
     </row>
-    <row r="133" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="133" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A133" t="s">
         <v>1220</v>
       </c>
@@ -36118,7 +36130,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="134" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="134" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A134" t="s">
         <v>825</v>
       </c>
@@ -36291,7 +36303,7 @@
         <v>42.1</v>
       </c>
     </row>
-    <row r="135" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="135" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A135" t="s">
         <v>1239</v>
       </c>
@@ -36461,7 +36473,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="136" spans="1:88" ht="44.1" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="136" spans="1:88" ht="44.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A136" t="s">
         <v>1250</v>
       </c>
@@ -36613,7 +36625,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="137" spans="1:88" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="137" spans="1:88" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A137" t="s">
         <v>1250</v>
       </c>
@@ -36777,7 +36789,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="138" spans="1:88" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="138" spans="1:88" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A138" t="s">
         <v>1265</v>
       </c>
@@ -36938,7 +36950,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="139" spans="1:88" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="139" spans="1:88" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A139" t="s">
         <v>1265</v>
       </c>
@@ -37096,7 +37108,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="140" spans="1:88" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="140" spans="1:88" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A140" t="s">
         <v>1265</v>
       </c>
@@ -37257,7 +37269,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="141" spans="1:88" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="141" spans="1:88" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A141" t="s">
         <v>1282</v>
       </c>
@@ -37430,7 +37442,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="142" spans="1:88" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="142" spans="1:88" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A142" t="s">
         <v>1293</v>
       </c>
@@ -37597,7 +37609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:88" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="143" spans="1:88" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A143" t="s">
         <v>1305</v>
       </c>
@@ -37791,7 +37803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:88" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="144" spans="1:88" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A144" t="s">
         <v>1318</v>
       </c>
@@ -37931,7 +37943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:88" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="145" spans="1:88" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A145" t="s">
         <v>1328</v>
       </c>
@@ -38132,13 +38144,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CJ145" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="National Supported Work Demonstration"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>